<commit_message>
feat: Martin reconcile, auth, PDF sprint (code without sample docs)
Push без docs/Люба и крупных бинарников — обход HTTP 408. Включает checkpoint aa5db07 и PDF sprint 2e37b63.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/server/fixtures/uk_card_mechel.xlsx
+++ b/server/fixtures/uk_card_mechel.xlsx
@@ -692,13 +692,13 @@
         <v>1083.50</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>117019539.25</v>
       </c>
       <c r="J8" t="str">
         <v>76.07.2</v>
       </c>
       <c r="K8" t="str">
-        <v/>
+        <v>Д</v>
       </c>
       <c r="L8" t="str">
         <v/>
@@ -736,7 +736,7 @@
         <v/>
       </c>
       <c r="K9" t="str">
-        <v/>
+        <v>Д</v>
       </c>
       <c r="L9" t="str">
         <v/>
@@ -769,13 +769,13 @@
         <v>61.00</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>117019600.25</v>
       </c>
       <c r="J10" t="str">
         <v>91.01.10</v>
       </c>
       <c r="K10" t="str">
-        <v/>
+        <v>Д</v>
       </c>
       <c r="L10" t="str">
         <v/>
@@ -813,7 +813,7 @@
         <v/>
       </c>
       <c r="K11" t="str">
-        <v/>
+        <v>Д</v>
       </c>
       <c r="L11" t="str">
         <v/>
@@ -846,13 +846,13 @@
         <v>97515.00</v>
       </c>
       <c r="I12" t="str">
-        <v/>
+        <v>117117115.25</v>
       </c>
       <c r="J12" t="str">
         <v>76.07.2</v>
       </c>
       <c r="K12" t="str">
-        <v/>
+        <v>Д</v>
       </c>
       <c r="L12" t="str">
         <v/>
@@ -884,13 +884,13 @@
         <v>5</v>
       </c>
       <c r="I13" t="str">
-        <v>17306736</v>
+        <v>17306741</v>
       </c>
       <c r="J13" t="str">
         <v/>
       </c>
       <c r="K13" t="str">
-        <v/>
+        <v>Д</v>
       </c>
       <c r="L13" t="str">
         <v/>

</xml_diff>